<commit_message>
WIP snapshot: review fixes in progress; holdout deal in review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLUCnhLjHTv59cWHgDLiCw
</commit_message>
<xml_diff>
--- a/qoe-evidence-review/data/holdout/kinetic_ridge_pt/adjustments/management_adjusted_ebitda.xlsx
+++ b/qoe-evidence-review/data/holdout/kinetic_ridge_pt/adjustments/management_adjusted_ebitda.xlsx
@@ -543,13 +543,13 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="5" t="n">
-        <v>3506181.68</v>
+        <v>3429088.66</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>3694433.98</v>
+        <v>3615913.06</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>3617050.4</v>
+        <v>3537376.14</v>
       </c>
     </row>
     <row r="8">
@@ -627,13 +627,13 @@
       <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="8" t="n">
-        <v>4214905.22</v>
+        <v>4137812.2</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>4433094.07</v>
+        <v>4354573.15</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>4361799.47</v>
+        <v>4282125.21</v>
       </c>
     </row>
     <row r="13">
@@ -736,7 +736,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>The Brownsburg clinic closed on February 27, 2026 and its lease was terminated effective March 31, 2026 for a $38,000 termination fee. Removes the clinic's operating results (legacy-billing revenue less clinic payroll, rent and utilities) and its closure costs (lease termination fee, legal, equipment move, final pay). Stranded shared costs (regional director, EMR enterprise license, billing office, employer taxes and benefits) are excluded.</t>
+          <t>The Brownsburg clinic closed on February 27, 2026 and its lease was terminated effective March 31, 2026 for a $38,250 termination fee. Removes the clinic's operating results (legacy-billing revenue less clinic payroll, rent and utilities) and its closure costs (lease termination fee, legal, equipment move, final pay). Stranded shared costs (regional director, EMR enterprise license, billing office, employer taxes and benefits) are excluded.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -756,7 +756,7 @@
         <v>177787.29</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>213222.46</v>
+        <v>213472.46</v>
       </c>
     </row>
     <row r="16">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Lease termination fee paid to Eagle Creek Commercial Properties under the March 2, 2026 lease termination agreement for the Brownsburg clinic ($38,000).</t>
+          <t>Lease termination fee paid to Eagle Creek Commercial Properties under the March 2, 2026 lease termination agreement for the Brownsburg clinic ($38,250).</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1248,7 +1248,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>38000</v>
+        <v>38250</v>
       </c>
     </row>
     <row r="28">
@@ -1306,7 +1306,7 @@
         <v>599063.29</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>1151548.46</v>
+        <v>1152048.46</v>
       </c>
     </row>
     <row r="31">
@@ -1321,13 +1321,13 @@
       <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr"/>
       <c r="G31" s="8" t="n">
-        <v>4469351.41</v>
+        <v>4392258.39</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>5032157.36</v>
+        <v>4953636.44</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>5513347.93</v>
+        <v>5434173.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>